<commit_message>
Add C4C, LockPhone, and Debt conso to the NPL type filter.
The sample data only had HP Home and HP Commercial, so those portfolios never appeared in the dropdown or charts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sample-data/dashboard-spec.xlsx
+++ b/sample-data/dashboard-spec.xlsx
@@ -22,9 +22,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSAT ซ่อม" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPL ภาพรวม'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NPL Stage'!$A$1:$E$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NPL ปิดสัญญา'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPL ภาพรวม'!$A$1:$D$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NPL Stage'!$A$1:$E$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NPL ปิดสัญญา'!$A$1:$H$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NPL HP Home 2568'!$A$1:$D$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ยอดขายสัดส่วน'!$A$1:$C$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ยอดขายสาขา'!$A$1:$D$41</definedName>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -523,113 +523,329 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="D4" t="n">
-        <v>42500000</v>
+        <v>9600000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>LockPhone</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5.4</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>18200000</v>
+        <v>6400000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>Debt conso</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3.9</v>
+        <v>7.2</v>
       </c>
       <c r="D6" t="n">
-        <v>42500000</v>
+        <v>11800000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>HP Home appliance</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5.4</v>
+        <v>3.9</v>
       </c>
       <c r="D7" t="n">
-        <v>18200000</v>
+        <v>42500000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>HP Commercial</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3.9</v>
+        <v>5.4</v>
       </c>
       <c r="D8" t="n">
-        <v>42500000</v>
+        <v>18200000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D9" t="n">
+        <v>9600000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>6400000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>11800000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>42500000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>18200000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D14" t="n">
+        <v>9600000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6400000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>11800000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Q3/2568</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D17" t="n">
+        <v>42500000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>HP Commercial</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C18" t="n">
         <v>5.4</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D18" t="n">
         <v>18200000</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>9600000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>6400000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>11800000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3046,7 +3262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3224,12 +3440,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3247,12 +3463,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3270,12 +3486,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3284,7 +3500,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="E10" t="n">
         <v>9800000</v>
@@ -3293,12 +3509,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>LockPhone</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3316,12 +3532,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>LockPhone</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3339,12 +3555,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>LockPhone</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3353,7 +3569,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>140</v>
+        <v>36</v>
       </c>
       <c r="E13" t="n">
         <v>9800000</v>
@@ -3362,12 +3578,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>Debt conso</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3385,12 +3601,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>Debt conso</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3408,12 +3624,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>Debt conso</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3422,7 +3638,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="E16" t="n">
         <v>9800000</v>
@@ -3431,12 +3647,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>HP Home appliance</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3454,12 +3670,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>HP Home appliance</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3477,12 +3693,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>HP Home appliance</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3491,7 +3707,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>140</v>
+        <v>95</v>
       </c>
       <c r="E19" t="n">
         <v>9800000</v>
@@ -3500,12 +3716,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>HP Commercial</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3523,12 +3739,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>HP Commercial</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3546,12 +3762,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>HP Commercial</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3560,7 +3776,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>95</v>
+        <v>140</v>
       </c>
       <c r="E22" t="n">
         <v>9800000</v>
@@ -3569,12 +3785,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3592,12 +3808,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3615,12 +3831,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3629,14 +3845,842 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>140</v>
+        <v>48</v>
       </c>
       <c r="E25" t="n">
         <v>9800000</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>820</v>
+      </c>
+      <c r="E26" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>210</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>36</v>
+      </c>
+      <c r="E28" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>820</v>
+      </c>
+      <c r="E29" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>210</v>
+      </c>
+      <c r="E30" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Q1/2568</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>72</v>
+      </c>
+      <c r="E31" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>820</v>
+      </c>
+      <c r="E32" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>210</v>
+      </c>
+      <c r="E33" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>95</v>
+      </c>
+      <c r="E34" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>820</v>
+      </c>
+      <c r="E35" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>210</v>
+      </c>
+      <c r="E36" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>140</v>
+      </c>
+      <c r="E37" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>820</v>
+      </c>
+      <c r="E38" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>210</v>
+      </c>
+      <c r="E39" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>48</v>
+      </c>
+      <c r="E40" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>820</v>
+      </c>
+      <c r="E41" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>210</v>
+      </c>
+      <c r="E42" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>36</v>
+      </c>
+      <c r="E43" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>820</v>
+      </c>
+      <c r="E44" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>210</v>
+      </c>
+      <c r="E45" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>72</v>
+      </c>
+      <c r="E46" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>820</v>
+      </c>
+      <c r="E47" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>210</v>
+      </c>
+      <c r="E48" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>95</v>
+      </c>
+      <c r="E49" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>820</v>
+      </c>
+      <c r="E50" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>210</v>
+      </c>
+      <c r="E51" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>140</v>
+      </c>
+      <c r="E52" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>820</v>
+      </c>
+      <c r="E53" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>210</v>
+      </c>
+      <c r="E54" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>48</v>
+      </c>
+      <c r="E55" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>820</v>
+      </c>
+      <c r="E56" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>210</v>
+      </c>
+      <c r="E57" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>36</v>
+      </c>
+      <c r="E58" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>820</v>
+      </c>
+      <c r="E59" t="n">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>210</v>
+      </c>
+      <c r="E60" t="n">
+        <v>7400000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>72</v>
+      </c>
+      <c r="E61" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E25"/>
+  <autoFilter ref="A1:E61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3647,7 +4691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3770,7 +4814,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>สินเชื่อเช่าซื้ออื่น</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3795,12 +4839,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>LockPhone</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -3825,12 +4869,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q1/2568</t>
+          <t>Q4/2567</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>Debt conso</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3860,7 +4904,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>สินเชื่อเช่าซื้ออื่น</t>
+          <t>HP Home appliance</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -3885,12 +4929,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>HP Commercial</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -3915,12 +4959,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>C4C</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -3945,12 +4989,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Q2/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>สินเชื่อเช่าซื้ออื่น</t>
+          <t>LockPhone</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -3975,12 +5019,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q1/2568</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HP Home appliance</t>
+          <t>Debt conso</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -4005,12 +5049,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q2/2568</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HP Commercial</t>
+          <t>HP Home appliance</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -4035,12 +5079,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Q3/2568</t>
+          <t>Q2/2568</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>สินเชื่อเช่าซื้ออื่น</t>
+          <t>HP Commercial</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -4062,8 +5106,248 @@
         <v>9800000</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G14" t="n">
+        <v>64</v>
+      </c>
+      <c r="H14" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G15" t="n">
+        <v>64</v>
+      </c>
+      <c r="H15" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Q2/2568</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>12</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G16" t="n">
+        <v>64</v>
+      </c>
+      <c r="H16" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HP Home appliance</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G17" t="n">
+        <v>64</v>
+      </c>
+      <c r="H17" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HP Commercial</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E18" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G18" t="n">
+        <v>64</v>
+      </c>
+      <c r="H18" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C4C</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E19" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G19" t="n">
+        <v>64</v>
+      </c>
+      <c r="H19" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LockPhone</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E20" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G20" t="n">
+        <v>64</v>
+      </c>
+      <c r="H20" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Q3/2568</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Debt conso</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E21" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="G21" t="n">
+        <v>64</v>
+      </c>
+      <c r="H21" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Show each NPL stage as grouped bars by quarter.
The stage chart previously summed every quarter into one bar, so the 2567 baseline could not be compared with later periods.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sample-data/dashboard-spec.xlsx
+++ b/sample-data/dashboard-spec.xlsx
@@ -3316,7 +3316,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>820</v>
+        <v>900</v>
       </c>
       <c r="E2" t="n">
         <v>12000000</v>
@@ -3339,7 +3339,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="E3" t="n">
         <v>7400000</v>
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E4" t="n">
         <v>9800000</v>
@@ -3385,7 +3385,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>820</v>
+        <v>900</v>
       </c>
       <c r="E5" t="n">
         <v>12000000</v>
@@ -3408,7 +3408,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="E6" t="n">
         <v>7400000</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="E7" t="n">
         <v>9800000</v>
@@ -3454,7 +3454,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>820</v>
+        <v>900</v>
       </c>
       <c r="E8" t="n">
         <v>12000000</v>
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="E9" t="n">
         <v>7400000</v>
@@ -3500,7 +3500,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="E10" t="n">
         <v>9800000</v>
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>820</v>
+        <v>900</v>
       </c>
       <c r="E11" t="n">
         <v>12000000</v>
@@ -3546,7 +3546,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="E12" t="n">
         <v>7400000</v>
@@ -3569,7 +3569,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="E13" t="n">
         <v>9800000</v>
@@ -3592,7 +3592,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>820</v>
+        <v>900</v>
       </c>
       <c r="E14" t="n">
         <v>12000000</v>
@@ -3615,7 +3615,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>210</v>
+        <v>180</v>
       </c>
       <c r="E15" t="n">
         <v>7400000</v>
@@ -3638,7 +3638,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E16" t="n">
         <v>9800000</v>
@@ -3661,10 +3661,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>820</v>
+        <v>745</v>
       </c>
       <c r="E17" t="n">
-        <v>12000000</v>
+        <v>11600000</v>
       </c>
     </row>
     <row r="18">
@@ -3684,10 +3684,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="E18" t="n">
-        <v>7400000</v>
+        <v>7650000</v>
       </c>
     </row>
     <row r="19">
@@ -3707,10 +3707,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="E19" t="n">
-        <v>9800000</v>
+        <v>9980000</v>
       </c>
     </row>
     <row r="20">
@@ -3730,10 +3730,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>820</v>
+        <v>745</v>
       </c>
       <c r="E20" t="n">
-        <v>12000000</v>
+        <v>11600000</v>
       </c>
     </row>
     <row r="21">
@@ -3753,10 +3753,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="E21" t="n">
-        <v>7400000</v>
+        <v>7650000</v>
       </c>
     </row>
     <row r="22">
@@ -3776,10 +3776,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="E22" t="n">
-        <v>9800000</v>
+        <v>9980000</v>
       </c>
     </row>
     <row r="23">
@@ -3799,10 +3799,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>820</v>
+        <v>745</v>
       </c>
       <c r="E23" t="n">
-        <v>12000000</v>
+        <v>11600000</v>
       </c>
     </row>
     <row r="24">
@@ -3822,10 +3822,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="E24" t="n">
-        <v>7400000</v>
+        <v>7650000</v>
       </c>
     </row>
     <row r="25">
@@ -3845,10 +3845,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="E25" t="n">
-        <v>9800000</v>
+        <v>9980000</v>
       </c>
     </row>
     <row r="26">
@@ -3868,10 +3868,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>820</v>
+        <v>745</v>
       </c>
       <c r="E26" t="n">
-        <v>12000000</v>
+        <v>11600000</v>
       </c>
     </row>
     <row r="27">
@@ -3891,10 +3891,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="E27" t="n">
-        <v>7400000</v>
+        <v>7650000</v>
       </c>
     </row>
     <row r="28">
@@ -3914,10 +3914,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="E28" t="n">
-        <v>9800000</v>
+        <v>9980000</v>
       </c>
     </row>
     <row r="29">
@@ -3937,10 +3937,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>820</v>
+        <v>745</v>
       </c>
       <c r="E29" t="n">
-        <v>12000000</v>
+        <v>11600000</v>
       </c>
     </row>
     <row r="30">
@@ -3960,10 +3960,10 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="E30" t="n">
-        <v>7400000</v>
+        <v>7650000</v>
       </c>
     </row>
     <row r="31">
@@ -3983,10 +3983,10 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E31" t="n">
-        <v>9800000</v>
+        <v>9980000</v>
       </c>
     </row>
     <row r="32">
@@ -4006,10 +4006,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>820</v>
+        <v>710</v>
       </c>
       <c r="E32" t="n">
-        <v>12000000</v>
+        <v>11200000</v>
       </c>
     </row>
     <row r="33">
@@ -4029,10 +4029,10 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>210</v>
+        <v>256</v>
       </c>
       <c r="E33" t="n">
-        <v>7400000</v>
+        <v>7900000</v>
       </c>
     </row>
     <row r="34">
@@ -4052,10 +4052,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E34" t="n">
-        <v>9800000</v>
+        <v>10160000</v>
       </c>
     </row>
     <row r="35">
@@ -4075,10 +4075,10 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>820</v>
+        <v>710</v>
       </c>
       <c r="E35" t="n">
-        <v>12000000</v>
+        <v>11200000</v>
       </c>
     </row>
     <row r="36">
@@ -4098,10 +4098,10 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>210</v>
+        <v>256</v>
       </c>
       <c r="E36" t="n">
-        <v>7400000</v>
+        <v>7900000</v>
       </c>
     </row>
     <row r="37">
@@ -4121,10 +4121,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="E37" t="n">
-        <v>9800000</v>
+        <v>10160000</v>
       </c>
     </row>
     <row r="38">
@@ -4144,10 +4144,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>820</v>
+        <v>710</v>
       </c>
       <c r="E38" t="n">
-        <v>12000000</v>
+        <v>11200000</v>
       </c>
     </row>
     <row r="39">
@@ -4167,10 +4167,10 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>210</v>
+        <v>256</v>
       </c>
       <c r="E39" t="n">
-        <v>7400000</v>
+        <v>7900000</v>
       </c>
     </row>
     <row r="40">
@@ -4190,10 +4190,10 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="E40" t="n">
-        <v>9800000</v>
+        <v>10160000</v>
       </c>
     </row>
     <row r="41">
@@ -4213,10 +4213,10 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>820</v>
+        <v>710</v>
       </c>
       <c r="E41" t="n">
-        <v>12000000</v>
+        <v>11200000</v>
       </c>
     </row>
     <row r="42">
@@ -4236,10 +4236,10 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>210</v>
+        <v>256</v>
       </c>
       <c r="E42" t="n">
-        <v>7400000</v>
+        <v>7900000</v>
       </c>
     </row>
     <row r="43">
@@ -4259,10 +4259,10 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="E43" t="n">
-        <v>9800000</v>
+        <v>10160000</v>
       </c>
     </row>
     <row r="44">
@@ -4282,10 +4282,10 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>820</v>
+        <v>710</v>
       </c>
       <c r="E44" t="n">
-        <v>12000000</v>
+        <v>11200000</v>
       </c>
     </row>
     <row r="45">
@@ -4305,10 +4305,10 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>210</v>
+        <v>256</v>
       </c>
       <c r="E45" t="n">
-        <v>7400000</v>
+        <v>7900000</v>
       </c>
     </row>
     <row r="46">
@@ -4328,10 +4328,10 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E46" t="n">
-        <v>9800000</v>
+        <v>10160000</v>
       </c>
     </row>
     <row r="47">
@@ -4351,10 +4351,10 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>820</v>
+        <v>675</v>
       </c>
       <c r="E47" t="n">
-        <v>12000000</v>
+        <v>10800000</v>
       </c>
     </row>
     <row r="48">
@@ -4374,10 +4374,10 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>210</v>
+        <v>274</v>
       </c>
       <c r="E48" t="n">
-        <v>7400000</v>
+        <v>8150000</v>
       </c>
     </row>
     <row r="49">
@@ -4397,10 +4397,10 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="E49" t="n">
-        <v>9800000</v>
+        <v>10340000</v>
       </c>
     </row>
     <row r="50">
@@ -4420,10 +4420,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>820</v>
+        <v>675</v>
       </c>
       <c r="E50" t="n">
-        <v>12000000</v>
+        <v>10800000</v>
       </c>
     </row>
     <row r="51">
@@ -4443,10 +4443,10 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>210</v>
+        <v>274</v>
       </c>
       <c r="E51" t="n">
-        <v>7400000</v>
+        <v>8150000</v>
       </c>
     </row>
     <row r="52">
@@ -4466,10 +4466,10 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="E52" t="n">
-        <v>9800000</v>
+        <v>10340000</v>
       </c>
     </row>
     <row r="53">
@@ -4489,10 +4489,10 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>820</v>
+        <v>675</v>
       </c>
       <c r="E53" t="n">
-        <v>12000000</v>
+        <v>10800000</v>
       </c>
     </row>
     <row r="54">
@@ -4512,10 +4512,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>210</v>
+        <v>274</v>
       </c>
       <c r="E54" t="n">
-        <v>7400000</v>
+        <v>8150000</v>
       </c>
     </row>
     <row r="55">
@@ -4535,10 +4535,10 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="E55" t="n">
-        <v>9800000</v>
+        <v>10340000</v>
       </c>
     </row>
     <row r="56">
@@ -4558,10 +4558,10 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>820</v>
+        <v>675</v>
       </c>
       <c r="E56" t="n">
-        <v>12000000</v>
+        <v>10800000</v>
       </c>
     </row>
     <row r="57">
@@ -4581,10 +4581,10 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>210</v>
+        <v>274</v>
       </c>
       <c r="E57" t="n">
-        <v>7400000</v>
+        <v>8150000</v>
       </c>
     </row>
     <row r="58">
@@ -4604,10 +4604,10 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="E58" t="n">
-        <v>9800000</v>
+        <v>10340000</v>
       </c>
     </row>
     <row r="59">
@@ -4627,10 +4627,10 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>820</v>
+        <v>675</v>
       </c>
       <c r="E59" t="n">
-        <v>12000000</v>
+        <v>10800000</v>
       </c>
     </row>
     <row r="60">
@@ -4650,10 +4650,10 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>210</v>
+        <v>274</v>
       </c>
       <c r="E60" t="n">
-        <v>7400000</v>
+        <v>8150000</v>
       </c>
     </row>
     <row r="61">
@@ -4673,10 +4673,10 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="E61" t="n">
-        <v>9800000</v>
+        <v>10340000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>